<commit_message>
Updated COL model - 2025-11-25 13:32
</commit_message>
<xml_diff>
--- a/VerveStacks_COL/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_COL/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_COL\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7F5CF58-ABE3-4BA0-8764-5F59D870C241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{089295F7-09E1-4D64-8F60-EEBDC4AEB9A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5942,7 +5942,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C4943E6-C4BC-4FB8-8765-5245A74229A6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DC32E8B-FCEB-402F-9FD8-2246AA0F7CDE}">
   <dimension ref="B9:M44"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7185,7 +7185,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15F66601-894A-47D9-8441-ECF9821F621B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E7D200A-03A5-4DE2-BB40-3B888D198E03}">
   <dimension ref="B9:Z20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -7957,7 +7957,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C211B47E-71A0-4FEC-AB7E-D4179FE23459}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{432E80A7-553B-428E-9A01-2EF18525AF9F}">
   <dimension ref="B9:P61"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>